<commit_message>
paper run 2026-09-01 11:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-01.xlsx
+++ b/reports/2026-09-01.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -681,13 +681,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>56.76</v>
+        <v>50.74</v>
       </c>
       <c r="E15" t="n">
         <v>8.93</v>
@@ -745,13 +745,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>12.23</v>
+        <v>6.21</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" t="n">
         <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>40.49</v>
+        <v>22.95</v>
       </c>
       <c r="E23" t="n">
         <v>8.93</v>
@@ -824,43 +824,43 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>12.23</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>30.11</v>
+        <v>12.23</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -869,254 +869,273 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>24.09</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" t="n">
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
         <v>14.42</v>
       </c>
-      <c r="E27" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="E28" t="n">
+        <v>8.93</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>15m</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>0.55–0.60</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>0.12–0.15%</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
         <v>8.93</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-09-01 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-01.xlsx
+++ b/reports/2026-09-01.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,49 @@
       </c>
       <c r="K2" t="n">
         <v>8.93</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-01T13:43:17.572290+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F3" t="n">
+        <v>18.79</v>
+      </c>
+      <c r="G3" t="n">
+        <v>36.14</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.00134</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>17.35</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +603,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8.93</v>
+        <v>26.28</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +643,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8.93</v>
+        <v>26.28</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>375.8099999999999</v>
+        <v>393.16</v>
       </c>
     </row>
     <row r="12">
@@ -681,77 +724,77 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>50.74</v>
+        <v>49.44</v>
       </c>
       <c r="E15" t="n">
-        <v>8.93</v>
+        <v>26.28</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>58.21</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>14.42</v>
-      </c>
-      <c r="E17" t="n">
-        <v>8.93</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>13.84</v>
+        <v>31.77</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>26.28</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>6.21</v>
+        <v>-5.82</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -760,17 +803,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>16.27</v>
+        <v>44.66</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -779,107 +822,107 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>37.04</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="n">
-        <v>16.27</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>22.95</v>
+        <v>90.95999999999999</v>
       </c>
       <c r="E23" t="n">
-        <v>8.93</v>
+        <v>17.35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>11.52</v>
+        <v>5.17</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>8.93</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>11.52</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
-        <v>12.23</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>24.09</v>
+        <v>12.23</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -888,207 +931,220 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>10</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>63.65</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" t="n">
-        <v>14.42</v>
-      </c>
-      <c r="E28" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>31.77</v>
+      </c>
+      <c r="E29" t="n">
+        <v>26.28</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>26.28</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>15m</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>26.28</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
         <v>8.93</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>17.35</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
-        <v>8.93</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>17.35</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1104,7 +1160,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По силе движения</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1126,17 +1182,55 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>26.28</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>8.93</v>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
+        <v>26.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-01 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-01.xlsx
+++ b/reports/2026-09-01.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,221 @@
       </c>
       <c r="K3" t="n">
         <v>17.35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-01T18:33:46.993907+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F4" t="n">
+        <v>19.66</v>
+      </c>
+      <c r="G4" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00214</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>16.74</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-01T22:48:46.947297+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>40.19</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00115</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>19.69</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-01T22:56:16.697070+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F6" t="n">
+        <v>21.48</v>
+      </c>
+      <c r="G6" t="n">
+        <v>42.12</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00148</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>20.64</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-01T23:03:47.286597+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F7" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="G7" t="n">
+        <v>44.14</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.00115</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>21.63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-01T23:11:42.368618+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00105</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>9.800000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +808,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +818,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -633,7 +848,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26.28</v>
+        <v>114.78</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +858,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>26.28</v>
+        <v>114.78</v>
       </c>
     </row>
     <row r="8">
@@ -673,7 +888,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>393.16</v>
+        <v>481.66</v>
       </c>
     </row>
     <row r="12">
@@ -724,16 +939,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>49.44</v>
+        <v>211.49</v>
       </c>
       <c r="E15" t="n">
-        <v>26.28</v>
+        <v>56.72</v>
       </c>
     </row>
     <row r="16">
@@ -743,16 +958,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>58.21</v>
+        <v>151.64</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>58.06</v>
       </c>
     </row>
     <row r="17">
@@ -769,16 +984,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>31.77</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>26.28</v>
+        <v>66.61</v>
       </c>
     </row>
     <row r="19">
@@ -788,13 +1003,13 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
         <v>2</v>
       </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
       <c r="D19" t="n">
-        <v>-5.82</v>
+        <v>14.01</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -807,16 +1022,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>44.66</v>
+        <v>137.81</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -826,16 +1041,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D21" t="n">
-        <v>37.04</v>
+        <v>139.21</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>38.37</v>
       </c>
     </row>
     <row r="22">
@@ -852,16 +1067,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C23" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D23" t="n">
-        <v>90.95999999999999</v>
+        <v>318.23</v>
       </c>
       <c r="E23" t="n">
-        <v>17.35</v>
+        <v>105.85</v>
       </c>
     </row>
     <row r="24">
@@ -871,13 +1086,13 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" t="n">
         <v>5</v>
       </c>
-      <c r="C24" t="n">
-        <v>3</v>
-      </c>
       <c r="D24" t="n">
-        <v>5.17</v>
+        <v>33.38</v>
       </c>
       <c r="E24" t="n">
         <v>8.93</v>
@@ -916,13 +1131,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D27" t="n">
-        <v>12.23</v>
+        <v>117.64</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -935,13 +1150,13 @@
         </is>
       </c>
       <c r="B28" t="n">
+        <v>13</v>
+      </c>
+      <c r="C28" t="n">
         <v>10</v>
       </c>
-      <c r="C28" t="n">
-        <v>7</v>
-      </c>
       <c r="D28" t="n">
-        <v>63.65</v>
+        <v>112.35</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -954,16 +1169,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D29" t="n">
-        <v>31.77</v>
+        <v>133.14</v>
       </c>
       <c r="E29" t="n">
-        <v>26.28</v>
+        <v>114.78</v>
       </c>
     </row>
     <row r="31">
@@ -1002,133 +1217,143 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>26.28</v>
+        <v>66.61</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>38.37</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>2</v>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" t="n">
-        <v>26.28</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>56.72</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>8.93</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
-        <v>17.35</v>
+        <v>58.06</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>8.93</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1144,7 +1369,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1154,83 +1379,217 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>8.93</v>
+        <v>16.74</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>40.33</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>31.43</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>2</v>
-      </c>
-      <c r="C48" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" t="n">
-        <v>26.28</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>6</v>
+      </c>
+      <c r="C50" t="n">
+        <v>6</v>
+      </c>
+      <c r="D50" t="n">
+        <v>105.85</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>8.93</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>51.12</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="n">
+        <v>3</v>
+      </c>
+      <c r="D55" t="n">
+        <v>46.92</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>16.74</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="n">
-        <v>26.28</v>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>43.02</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="n">
+        <v>71.76000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>